<commit_message>
Se agrega opcion Si,No en anticipos
</commit_message>
<xml_diff>
--- a/DataTables/FACTURACION/EmitirFacturaFoa.xlsx
+++ b/DataTables/FACTURACION/EmitirFacturaFoa.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="903" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="903" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,11 +20,11 @@
     <sheet name="Padrones" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'conceptoRecuperos'!$A$1:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'conceptoRecuperos'!$A$1:$M$34</definedName>
   </definedNames>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache cacheId="52" r:id="rId13"/>
+    <pivotCache cacheId="19" r:id="rId13"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -127,12 +127,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.7999816888943144"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -178,6 +172,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="65"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -194,13 +194,13 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
@@ -215,20 +215,20 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
@@ -242,30 +242,27 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="1" xfId="1"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="1" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="1" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="38">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -307,7 +304,97 @@
     <cellStyle name="Moneda 4 3" xfId="36"/>
     <cellStyle name="Moneda 5 2" xfId="37"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color theme="1"/>
+        <extend val="0"/>
+        <sz val="11"/>
+        <vertAlign val="baseline"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom"/>
+      <border outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color theme="1"/>
+        <extend val="0"/>
+        <sz val="11"/>
+        <vertAlign val="baseline"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom"/>
+      <border outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <condense val="0"/>
+        <color theme="1"/>
+        <extend val="0"/>
+        <sz val="11"/>
+        <vertAlign val="baseline"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+      <fill>
+        <patternFill>
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom"/>
+      <border outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -412,9 +499,9 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshedBy="Pablo" refreshedDate="45484.41388530093" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="28" r:id="rId1">
+<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshedBy="Pablo" refreshedDate="45790.95587824074" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="34" r:id="rId1">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:M29" sheet="conceptoRecuperos"/>
+    <worksheetSource ref="A1:M35" sheet="conceptoRecuperos"/>
   </cacheSource>
   <cacheFields count="13">
     <cacheField name="i_factura" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
@@ -437,7 +524,7 @@
       <sharedItems count="0"/>
     </cacheField>
     <cacheField name="i_netoGravado" uniqueList="1" numFmtId="49" sqlType="0" hierarchy="0" level="0" databaseField="1">
-      <sharedItems count="0" containsBlank="1"/>
+      <sharedItems count="0" containsBlank="1" containsNumber="1" containsString="0" minValue="44257.72400323056" maxValue="18959178.56800465"/>
     </cacheField>
     <cacheField name="i_descripcion" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0"/>
@@ -452,452 +539,542 @@
       <sharedItems count="0"/>
     </cacheField>
     <cacheField name="formatoNumero" uniqueList="1" numFmtId="44" sqlType="0" hierarchy="0" level="0" databaseField="1">
-      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="1166987.15"/>
+      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="18959178.56800465"/>
     </cacheField>
     <cacheField name="IVA21" uniqueList="1" numFmtId="44" sqlType="0" hierarchy="0" level="0" databaseField="1">
-      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="55264.9314"/>
+      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="142743.6409588355"/>
     </cacheField>
     <cacheField name="IVA27" uniqueList="1" numFmtId="44" sqlType="0" hierarchy="0" level="0" databaseField="1">
-      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="315086.5305"/>
+      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="5118978.213361257"/>
     </cacheField>
     <cacheField name="Final" uniqueList="1" numFmtId="44" sqlType="0" hierarchy="0" level="0" databaseField="1">
-      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="1482073.6805"/>
+      <sharedItems count="0" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="24078156.78136591"/>
     </cacheField>
   </cacheFields>
 </pivotCacheDefinition>
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34">
   <r>
     <s v="SI"/>
     <x v="0"/>
     <s v="CONSUMO DE AGUA"/>
     <s v="IVA (27%)"/>
-    <s v="1166987,15"/>
+    <n v="18959178.56800465"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="1166987.15"/>
-    <n v="0"/>
-    <n v="315086.5305"/>
-    <n v="1482073.6805"/>
+    <n v="18959178.56800465"/>
+    <n v="0"/>
+    <n v="5118978.213361257"/>
+    <n v="24078156.78136591"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="0"/>
     <s v="GENERAL"/>
     <s v="IVA (21%)"/>
-    <s v="240373,17"/>
+    <n v="187444.4781313295"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="240373.17"/>
-    <n v="50478.3657"/>
-    <n v="0"/>
-    <n v="290851.5357"/>
+    <n v="187444.4781313295"/>
+    <n v="39363.34040757919"/>
+    <n v="0"/>
+    <n v="226807.8185389087"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="0"/>
     <s v="LA INDIA"/>
     <s v="IVA (21%)"/>
-    <s v="263166,34"/>
+    <n v="679731.6236135026"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="263166.34"/>
-    <n v="55264.9314"/>
-    <n v="0"/>
-    <n v="318431.2714"/>
+    <n v="679731.6236135026"/>
+    <n v="142743.6409588355"/>
+    <n v="0"/>
+    <n v="822475.2645723382"/>
+  </r>
+  <r>
+    <s v="NO"/>
+    <x v="0"/>
+    <s v="POZO 2"/>
+    <s v="IVA (21%)"/>
+    <m/>
+    <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
+    <s v="Concepto"/>
+    <n v="1"/>
+    <s v="418001002"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="1"/>
     <s v="AGUA POZO 1"/>
     <s v="IVA (27%)"/>
-    <s v="104278,80"/>
+    <n v="319384.9009558766"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="104278.8"/>
-    <n v="0"/>
-    <n v="28155.276"/>
-    <n v="132434.076"/>
+    <n v="319384.9009558766"/>
+    <n v="0"/>
+    <n v="86233.92325808668"/>
+    <n v="405618.8242139632"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="1"/>
     <s v="AGUA POZO 3"/>
     <s v="IVA (27%)"/>
-    <s v="107348,41"/>
+    <n v="409240.0481302512"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="107348.41"/>
-    <n v="0"/>
-    <n v="28984.0707"/>
-    <n v="136332.4807"/>
+    <n v="409240.0481302512"/>
+    <n v="0"/>
+    <n v="110494.8129951678"/>
+    <n v="519734.8611254191"/>
   </r>
   <r>
-    <s v="SI"/>
+    <s v="NO"/>
     <x v="1"/>
     <s v="CONSUMO DE AGUA"/>
     <s v="IVA (27%)"/>
-    <s v="1000964,87"/>
+    <m/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="1000964.87"/>
-    <n v="0"/>
-    <n v="270260.5149"/>
-    <n v="1271225.3849"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="1"/>
     <s v="GENERAL"/>
     <s v="IVA (21%)"/>
-    <s v="192298,54"/>
+    <n v="149955.5825050636"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="192298.54"/>
-    <n v="40382.6934"/>
-    <n v="0"/>
-    <n v="232681.2334"/>
+    <n v="149955.5825050636"/>
+    <n v="31490.67232606335"/>
+    <n v="0"/>
+    <n v="181446.2548311269"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="1"/>
     <s v="LA INDIA"/>
     <s v="IVA (21%)"/>
-    <s v="210533,07"/>
+    <n v="543785.2988908022"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="210533.07"/>
-    <n v="44211.9447"/>
-    <n v="0"/>
-    <n v="254745.0147"/>
+    <n v="543785.2988908022"/>
+    <n v="114194.9127670685"/>
+    <n v="0"/>
+    <n v="657980.2116578707"/>
+  </r>
+  <r>
+    <s v="NO"/>
+    <x v="1"/>
+    <s v="POZO 3"/>
+    <s v="IVA (21%)"/>
+    <m/>
+    <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
+    <s v="Concepto"/>
+    <n v="1"/>
+    <s v="418001002"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="2"/>
     <s v="AGUA POZO 1"/>
     <s v="IVA (27%)"/>
-    <s v="177077,20"/>
+    <n v="838874.4163529938"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="177077.2"/>
-    <n v="0"/>
-    <n v="47810.844"/>
-    <n v="224888.044"/>
+    <n v="838874.4163529938"/>
+    <n v="0"/>
+    <n v="226496.0924153083"/>
+    <n v="1065370.508768302"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="2"/>
     <s v="AGUA POZO 3"/>
     <s v="IVA (27%)"/>
-    <s v="182289,75"/>
+    <n v="1153726.931152588"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="182289.75"/>
-    <n v="0"/>
-    <n v="49218.23250000001"/>
-    <n v="231507.9825"/>
+    <n v="1153726.931152588"/>
+    <n v="0"/>
+    <n v="311506.2714111987"/>
+    <n v="1465233.202563786"/>
   </r>
   <r>
-    <s v="SI"/>
+    <s v="NO"/>
     <x v="2"/>
     <s v="CONSUMO DE AGUA"/>
     <s v="IVA (27%)"/>
-    <s v="845270,15"/>
+    <m/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="845270.15"/>
-    <n v="0"/>
-    <n v="228222.9405"/>
-    <n v="1073493.0905"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="2"/>
     <s v="GENERAL"/>
     <s v="IVA (21%)"/>
-    <s v="116029,46"/>
+    <n v="90480.49095220458"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="116029.46"/>
-    <n v="24366.1866"/>
-    <n v="0"/>
-    <n v="140395.6466"/>
+    <n v="90480.49095220458"/>
+    <n v="19000.90309996296"/>
+    <n v="0"/>
+    <n v="109481.3940521675"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="2"/>
     <s v="LA INDIA"/>
     <s v="IVA (21%)"/>
-    <s v="127031,85"/>
+    <n v="328110.2310050356"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="127031.85"/>
-    <n v="26676.6885"/>
-    <n v="0"/>
-    <n v="153708.5385"/>
+    <n v="328110.2310050356"/>
+    <n v="68903.14851105749"/>
+    <n v="0"/>
+    <n v="397013.3795160931"/>
+  </r>
+  <r>
+    <s v="NO"/>
+    <x v="2"/>
+    <s v="POZO 1"/>
+    <s v="IVA (21%)"/>
+    <m/>
+    <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
+    <s v="Concepto"/>
+    <n v="1"/>
+    <s v="418001002"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="3"/>
     <s v="AGUA POZO 1"/>
     <s v="IVA (27%)"/>
-    <s v="69650,37"/>
+    <n v="745057.6481347701"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="69650.37"/>
-    <n v="0"/>
-    <n v="18805.5999"/>
-    <n v="88455.9699"/>
+    <n v="745057.6481347701"/>
+    <n v="0"/>
+    <n v="201165.564996388"/>
+    <n v="946223.213131158"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="3"/>
     <s v="AGUA POZO 3"/>
     <s v="IVA (27%)"/>
-    <s v="71700,63"/>
+    <n v="859343.9439895941"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="71700.63"/>
-    <n v="0"/>
-    <n v="19359.1701"/>
-    <n v="91059.80010000001"/>
+    <n v="859343.9439895941"/>
+    <n v="0"/>
+    <n v="232022.8648771904"/>
+    <n v="1091366.808866784"/>
   </r>
   <r>
-    <s v="SI"/>
+    <s v="NO"/>
     <x v="3"/>
     <s v="CONSUMO DE AGUA"/>
     <s v="IVA (27%)"/>
-    <s v="377594,89"/>
+    <m/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="377594.89"/>
-    <n v="0"/>
-    <n v="101950.6203"/>
-    <n v="479545.5103"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="3"/>
     <s v="GENERAL"/>
     <s v="IVA (21%)"/>
-    <s v="56754,78"/>
+    <n v="44257.72400323056"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="56754.78"/>
-    <n v="11918.5038"/>
-    <n v="0"/>
-    <n v="68673.2838"/>
+    <n v="44257.72400323056"/>
+    <n v="9294.122040678418"/>
+    <n v="0"/>
+    <n v="53551.84604390898"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="3"/>
     <s v="LA INDIA"/>
     <s v="IVA (21%)"/>
-    <s v="62136,50"/>
+    <n v="160492.1889087438"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="62136.5"/>
-    <n v="13048.665"/>
-    <n v="0"/>
-    <n v="75185.16499999999"/>
+    <n v="160492.1889087438"/>
+    <n v="33703.35967083619"/>
+    <n v="0"/>
+    <n v="194195.5485795799"/>
   </r>
   <r>
     <s v="NO"/>
+    <x v="3"/>
+    <s v="POZO 1"/>
+    <s v="IVA (21%)"/>
+    <m/>
+    <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
+    <s v="Concepto"/>
+    <n v="1"/>
+    <s v="418001002"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <s v="SI"/>
     <x v="4"/>
     <s v="AGUA POZO 1"/>
     <s v="IVA (27%)"/>
-    <m/>
+    <n v="1377109.545337181"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo: (AB)"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
+    <n v="1377109.545337181"/>
+    <n v="0"/>
+    <n v="371819.577241039"/>
+    <n v="1748929.12257822"/>
   </r>
   <r>
-    <s v="NO"/>
+    <s v="SI"/>
     <x v="4"/>
     <s v="AGUA POZO 3"/>
     <s v="IVA (27%)"/>
-    <m/>
+    <n v="638105.4135885102"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo: (AB)"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
+    <n v="638105.4135885102"/>
+    <n v="0"/>
+    <n v="172288.4616688978"/>
+    <n v="810393.875257408"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="4"/>
     <s v="CONSUMO DE AGUA"/>
     <s v="IVA (27%)"/>
-    <s v="281861,66"/>
+    <n v="105002.6994626316"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo: (AB)"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="281861.66"/>
-    <n v="0"/>
-    <n v="76102.6482"/>
-    <n v="357964.3082"/>
+    <n v="105002.6994626316"/>
+    <n v="0"/>
+    <n v="28350.72885491053"/>
+    <n v="133353.4283175421"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="4"/>
     <s v="GENERAL"/>
     <s v="IVA (21%)"/>
-    <s v="69441,14"/>
+    <n v="54150.62701571741"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="69441.14"/>
-    <n v="14582.6394"/>
-    <n v="0"/>
-    <n v="84023.7794"/>
+    <n v="54150.62701571741"/>
+    <n v="11371.63167330066"/>
+    <n v="0"/>
+    <n v="65522.25868901806"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="4"/>
     <s v="LA INDIA"/>
     <s v="IVA (21%)"/>
-    <s v="76025,83"/>
+    <n v="196366.9134883452"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="76025.83"/>
-    <n v="15965.4243"/>
-    <n v="0"/>
-    <n v="91991.2543"/>
+    <n v="196366.9134883452"/>
+    <n v="41237.05183255249"/>
+    <n v="0"/>
+    <n v="237603.9653208977"/>
+  </r>
+  <r>
+    <s v="NO"/>
+    <x v="4"/>
+    <s v="POZO 3"/>
+    <s v="IVA (21%)"/>
+    <m/>
+    <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)"/>
+    <s v="Concepto"/>
+    <n v="1"/>
+    <s v="418001002"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="5"/>
     <s v="AGUA POZO 1"/>
     <s v="IVA (27%)"/>
-    <s v="109394,36"/>
+    <n v="652413.0217518924"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="109394.36"/>
-    <n v="0"/>
-    <n v="29536.4772"/>
-    <n v="138930.8372"/>
+    <n v="652413.0217518924"/>
+    <n v="0"/>
+    <n v="176151.515873011"/>
+    <n v="828564.5376249034"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="5"/>
     <s v="AGUA POZO 3"/>
     <s v="IVA (27%)"/>
-    <s v="112614,55"/>
+    <n v="768120.0231390562"/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="112614.55"/>
-    <n v="0"/>
-    <n v="30405.9285"/>
-    <n v="143020.4785"/>
+    <n v="768120.0231390562"/>
+    <n v="0"/>
+    <n v="207392.4062475452"/>
+    <n v="975512.4293866013"/>
   </r>
   <r>
-    <s v="SI"/>
+    <s v="NO"/>
     <x v="5"/>
     <s v="CONSUMO DE AGUA"/>
     <s v="IVA (27%)"/>
-    <s v="491830,13"/>
+    <m/>
     <s v="RECUPERO ENERGIA ELECTRICA Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="491830.13"/>
-    <n v="0"/>
-    <n v="132794.1351"/>
-    <n v="624624.2651"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="5"/>
     <s v="GENERAL"/>
     <s v="IVA (21%)"/>
-    <s v="64201,00"/>
+    <n v="50064.33739245442"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="64201"/>
-    <n v="13482.21"/>
-    <n v="0"/>
-    <n v="77683.20999999999"/>
+    <n v="50064.33739245442"/>
+    <n v="10513.51085241543"/>
+    <n v="0"/>
+    <n v="60577.84824486985"/>
   </r>
   <r>
     <s v="SI"/>
     <x v="5"/>
     <s v="LA INDIA"/>
     <s v="IVA (21%)"/>
-    <s v="70288,81"/>
+    <n v="181548.7640935708"/>
     <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
     <s v="Concepto"/>
     <n v="1"/>
     <s v="418001002"/>
-    <n v="70288.81"/>
-    <n v="14760.6501"/>
-    <n v="0"/>
-    <n v="85049.4601"/>
+    <n v="181548.7640935708"/>
+    <n v="38125.24045964987"/>
+    <n v="0"/>
+    <n v="219674.0045532207"/>
+  </r>
+  <r>
+    <s v="NO"/>
+    <x v="5"/>
+    <s v="POZO 1"/>
+    <s v="IVA (21%)"/>
+    <m/>
+    <s v="RENDICIÓN GASTOS FIDEICOMISO Periodo:"/>
+    <s v="Concepto"/>
+    <n v="1"/>
+    <s v="418001002"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="52" dataOnRows="0" dataCaption="Valores" showError="0" showMissing="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="1" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="8" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="1" outline="1" outlineData="1" compactData="1" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="0" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
+<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="19" dataOnRows="0" dataCaption="Valores" showError="0" showMissing="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="1" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="8" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="1" outline="1" outlineData="1" compactData="1" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="0" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
-    <pivotField axis="axisRow" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
+    <pivotField axis="axisRow" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="ascending" defaultSubtotal="1">
       <items count="7">
         <item t="data" sd="1" x="0"/>
         <item t="data" sd="1" x="1"/>
@@ -953,7 +1130,7 @@
     <dataField name="Suma de Final" fld="12" subtotal="sum" showDataAs="normal" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format action="formatting" dxfId="0">
+    <format action="formatting" dxfId="3">
       <pivotArea type="normal" dataOnly="1" outline="1" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="1"/>
@@ -1269,7 +1446,7 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="31.140625" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
+    <col width="31.140625" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1321,8 +1498,8 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="21.85546875" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="21.85546875" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1376,8 +1553,8 @@
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="25.42578125" bestFit="1" customWidth="1" style="25" min="2" max="3"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="25.42578125" bestFit="1" customWidth="1" style="23" min="2" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1550,8 +1727,8 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="37.85546875" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="31" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
+    <col width="37.85546875" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="31" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1657,7 +1834,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">POZO 1  </t>
+          <t>POZO 1</t>
         </is>
       </c>
     </row>
@@ -1669,14 +1846,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">POZO 2  </t>
+          <t>POZO 2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">POZO 3  </t>
+          <t>POZO 3</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1867,7 @@
     <row r="10">
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">GENERAL  </t>
+          <t>GENERAL</t>
         </is>
       </c>
     </row>
@@ -1705,21 +1882,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="8.7109375" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="20.140625" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
-    <col width="10.7109375" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
-    <col width="16.140625" bestFit="1" customWidth="1" style="25" min="4" max="4"/>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="5" max="5"/>
-    <col width="12.7109375" bestFit="1" customWidth="1" style="25" min="6" max="6"/>
-    <col width="12" bestFit="1" customWidth="1" style="25" min="7" max="7"/>
-    <col width="16.5703125" bestFit="1" customWidth="1" style="25" min="8" max="8"/>
-    <col width="15" bestFit="1" customWidth="1" style="15" min="9" max="9"/>
+    <col width="8.7109375" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="20.140625" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
+    <col width="16.140625" bestFit="1" customWidth="1" style="23" min="4" max="4"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="5" max="5"/>
+    <col width="12.7109375" bestFit="1" customWidth="1" style="23" min="6" max="6"/>
+    <col width="12" bestFit="1" customWidth="1" style="23" min="7" max="7"/>
+    <col width="16" customWidth="1" style="23" min="8" max="8"/>
+    <col width="15" bestFit="1" customWidth="1" style="13" min="9" max="9"/>
     <col width="17.85546875" bestFit="1" customWidth="1" style="10" min="10" max="10"/>
-    <col width="10.140625" bestFit="1" customWidth="1" style="25" min="11" max="11"/>
-    <col width="13" bestFit="1" customWidth="1" style="13" min="12" max="12"/>
+    <col width="10.140625" bestFit="1" customWidth="1" style="23" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1763,7 +1939,7 @@
           <t>i_mesFacturacion</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>i_montoControl</t>
         </is>
@@ -1776,11 +1952,6 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>o_asiento</t>
-        </is>
-      </c>
-      <c r="L1" s="13" t="inlineStr">
-        <is>
-          <t>controlTablas</t>
         </is>
       </c>
     </row>
@@ -1797,12 +1968,12 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>30/06/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>0001-00000695</t>
+          <t>0001-00000727</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1822,26 +1993,23 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>06 / 2024</t>
-        </is>
-      </c>
-      <c r="I2" s="19" t="inlineStr">
-        <is>
-          <t>2091356</t>
+          <t>04 / 2025</t>
+        </is>
+      </c>
+      <c r="I2" s="17" t="inlineStr">
+        <is>
+          <t>25127439</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2091356</t>
+          <t>25127439</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5-VEN-10</t>
-        </is>
-      </c>
-      <c r="L2" s="27" t="n">
-        <v>998664.2556</v>
+          <t>5-VEN-94</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1857,12 +2025,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>30/06/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>0001-00000694</t>
+          <t>0001-00000725</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1882,26 +2050,23 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>06 / 2024</t>
-        </is>
-      </c>
-      <c r="I3" s="16" t="inlineStr">
-        <is>
-          <t>2027418</t>
+          <t>04 / 2025</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>1764780</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2027418</t>
+          <t>1764780</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>5-VEN-11</t>
-        </is>
-      </c>
-      <c r="L3" s="27" t="n">
-        <v>798931.4068999999</v>
+          <t>5-VEN-95</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1917,12 +2082,12 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>30/06/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>0001-00000690</t>
+          <t>0001-00000726</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1942,26 +2107,23 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>06 / 2024</t>
-        </is>
-      </c>
-      <c r="I4" s="19" t="inlineStr">
-        <is>
-          <t>1823993</t>
-        </is>
-      </c>
-      <c r="J4" s="17" t="inlineStr">
-        <is>
-          <t>1823993</t>
+          <t>04 / 2025</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>3037098</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>3037098</t>
         </is>
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>5-VEN-12</t>
-        </is>
-      </c>
-      <c r="L4" s="27" t="n">
-        <v>482060.7814</v>
+          <t>5-VEN-96</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1977,12 +2139,12 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>30/06/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>0001-00000692</t>
+          <t>0001-00000723</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2002,26 +2164,23 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>06 / 2024</t>
-        </is>
-      </c>
-      <c r="I5" s="19" t="inlineStr">
-        <is>
-          <t>802919</t>
-        </is>
-      </c>
-      <c r="J5" s="17" t="inlineStr">
-        <is>
-          <t>802919</t>
+          <t>04 / 2025</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>2285337</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>2285337</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>5-VEN-13</t>
-        </is>
-      </c>
-      <c r="L5" s="27" t="n">
-        <v>235795.725</v>
+          <t>5-VEN-97</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2037,12 +2196,12 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>30/06/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>0001-00000693</t>
+          <t>0001-00000724</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -2062,26 +2221,23 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>06 / 2024</t>
-        </is>
-      </c>
-      <c r="I6" s="16" t="inlineStr">
-        <is>
-          <t>533979</t>
+          <t>04 / 2025</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>2995802</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>533979</t>
+          <t>2995802</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>5-VEN-14</t>
-        </is>
-      </c>
-      <c r="L6" s="27" t="n">
-        <v>288502.9983</v>
+          <t>5-VEN-98</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -2097,12 +2253,12 @@
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>30/06/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>0001-00000691</t>
+          <t>0001-00000722</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2122,31 +2278,28 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>06 / 2024</t>
-        </is>
-      </c>
-      <c r="I7" s="15" t="inlineStr">
-        <is>
-          <t>1069308</t>
+          <t>04 / 2025</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>2084328</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1069308</t>
+          <t>2084328</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>5-VEN-15</t>
-        </is>
-      </c>
-      <c r="L7" s="27" t="n">
-        <v>266732.1217</v>
+          <t>5-VEN-99</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="E8" s="3" t="n"/>
-      <c r="I8" s="22" t="n"/>
+      <c r="I8" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="D10" s="3" t="n"/>
@@ -2155,11 +2308,8 @@
     <row r="11">
       <c r="D11" s="3" t="n"/>
     </row>
-    <row r="13">
-      <c r="E13" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="E15" s="3" t="n"/>
+    <row r="12">
+      <c r="D12" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2173,22 +2323,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col width="11" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
-    <col width="18.85546875" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
-    <col width="11.85546875" bestFit="1" customWidth="1" style="25" min="4" max="4"/>
-    <col width="16.28515625" bestFit="1" customWidth="1" style="10" min="5" max="5"/>
-    <col width="43.7109375" bestFit="1" customWidth="1" style="25" min="6" max="6"/>
-    <col width="12.5703125" bestFit="1" customWidth="1" style="25" min="7" max="7"/>
-    <col width="13" bestFit="1" customWidth="1" style="25" min="8" max="8"/>
-    <col width="19" bestFit="1" customWidth="1" style="25" min="9" max="9"/>
-    <col width="19.28515625" bestFit="1" customWidth="1" style="25" min="10" max="10"/>
-    <col width="12" bestFit="1" customWidth="1" style="25" min="11" max="11"/>
-    <col width="13" bestFit="1" customWidth="1" style="25" min="12" max="12"/>
-    <col width="14.5703125" bestFit="1" customWidth="1" style="25" min="13" max="13"/>
+    <col width="11" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.85546875" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
+    <col width="11.85546875" bestFit="1" customWidth="1" style="23" min="4" max="4"/>
+    <col width="16.7109375" bestFit="1" customWidth="1" style="10" min="5" max="5"/>
+    <col width="43.7109375" bestFit="1" customWidth="1" style="23" min="6" max="6"/>
+    <col width="12.5703125" bestFit="1" customWidth="1" style="23" min="7" max="7"/>
+    <col width="13" bestFit="1" customWidth="1" style="23" min="8" max="8"/>
+    <col width="19" bestFit="1" customWidth="1" style="23" min="9" max="9"/>
+    <col width="19.28515625" bestFit="1" customWidth="1" style="23" min="10" max="10"/>
+    <col width="14.5703125" bestFit="1" customWidth="1" style="23" min="11" max="12"/>
+    <col width="15.5703125" bestFit="1" customWidth="1" style="23" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2237,7 +2386,7 @@
           <t>i_cuentaContable</t>
         </is>
       </c>
-      <c r="J1" s="28" t="inlineStr">
+      <c r="J1" s="25" t="inlineStr">
         <is>
           <t>formatoNumero</t>
         </is>
@@ -2279,9 +2428,9 @@
           <t>IVA (27%)</t>
         </is>
       </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>1166987,15</t>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>18959178,5680047</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2302,19 +2451,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J2" s="28">
+      <c r="J2" s="25">
         <f>VALUE(E2)</f>
         <v/>
       </c>
-      <c r="K2" s="28">
+      <c r="K2" s="25">
         <f>IF(D2="IVA (21%)",J2*0.21,0)</f>
         <v/>
       </c>
-      <c r="L2" s="28">
+      <c r="L2" s="25">
         <f>IF(D2="IVA (27%)",J2*0.27,0)</f>
         <v/>
       </c>
-      <c r="M2" s="29">
+      <c r="M2" s="26">
         <f>SUM(J2:L2)</f>
         <v/>
       </c>
@@ -2340,9 +2489,9 @@
           <t>IVA (21%)</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
-        <is>
-          <t>240373,17</t>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>187444,478131329</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -2363,19 +2512,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J3" s="28">
+      <c r="J3" s="25">
         <f>VALUE(E3)</f>
         <v/>
       </c>
-      <c r="K3" s="28">
+      <c r="K3" s="25">
         <f>IF(D3="IVA (21%)",J3*0.21,0)</f>
         <v/>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="25">
         <f>IF(D3="IVA (27%)",J3*0.27,0)</f>
         <v/>
       </c>
-      <c r="M3" s="29">
+      <c r="M3" s="26">
         <f>SUM(J3:L3)</f>
         <v/>
       </c>
@@ -2401,9 +2550,9 @@
           <t>IVA (21%)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
-        <is>
-          <t>263166,34</t>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>679731,623613503</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -2424,19 +2573,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J4" s="28">
+      <c r="J4" s="25">
         <f>VALUE(E4)</f>
         <v/>
       </c>
-      <c r="K4" s="28">
+      <c r="K4" s="25">
         <f>IF(D4="IVA (21%)",J4*0.21,0)</f>
         <v/>
       </c>
-      <c r="L4" s="28">
+      <c r="L4" s="25">
         <f>IF(D4="IVA (27%)",J4*0.27,0)</f>
         <v/>
       </c>
-      <c r="M4" s="29">
+      <c r="M4" s="26">
         <f>SUM(J4:L4)</f>
         <v/>
       </c>
@@ -2444,32 +2593,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FINCAS Y BODEGAS MONTECHEZ S.A.</t>
+          <t>CABALGANDO SAFI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AGUA POZO 1</t>
+          <t>POZO 2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>104278,80</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2485,19 +2630,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J5" s="28">
+      <c r="J5" s="25">
         <f>VALUE(E5)</f>
         <v/>
       </c>
-      <c r="K5" s="28">
+      <c r="K5" s="25">
         <f>IF(D5="IVA (21%)",J5*0.21,0)</f>
         <v/>
       </c>
-      <c r="L5" s="28">
+      <c r="L5" s="25">
         <f>IF(D5="IVA (27%)",J5*0.27,0)</f>
         <v/>
       </c>
-      <c r="M5" s="29">
+      <c r="M5" s="26">
         <f>SUM(J5:L5)</f>
         <v/>
       </c>
@@ -2515,7 +2660,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AGUA POZO 3</t>
+          <t>AGUA POZO 1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2523,9 +2668,9 @@
           <t>IVA (27%)</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>107348,41</t>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>319384,900955877</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2546,19 +2691,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J6" s="28">
+      <c r="J6" s="25">
         <f>VALUE(E6)</f>
         <v/>
       </c>
-      <c r="K6" s="28">
+      <c r="K6" s="25">
         <f>IF(D6="IVA (21%)",J6*0.21,0)</f>
         <v/>
       </c>
-      <c r="L6" s="28">
+      <c r="L6" s="25">
         <f>IF(D6="IVA (27%)",J6*0.27,0)</f>
         <v/>
       </c>
-      <c r="M6" s="29">
+      <c r="M6" s="26">
         <f>SUM(J6:L6)</f>
         <v/>
       </c>
@@ -2576,7 +2721,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CONSUMO DE AGUA</t>
+          <t>AGUA POZO 3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2584,9 +2729,9 @@
           <t>IVA (27%)</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>1000964,87</t>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>409240,048130251</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2607,19 +2752,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J7" s="28">
+      <c r="J7" s="25">
         <f>VALUE(E7)</f>
         <v/>
       </c>
-      <c r="K7" s="28">
+      <c r="K7" s="25">
         <f>IF(D7="IVA (21%)",J7*0.21,0)</f>
         <v/>
       </c>
-      <c r="L7" s="28">
+      <c r="L7" s="25">
         <f>IF(D7="IVA (27%)",J7*0.27,0)</f>
         <v/>
       </c>
-      <c r="M7" s="29">
+      <c r="M7" s="26">
         <f>SUM(J7:L7)</f>
         <v/>
       </c>
@@ -2627,7 +2772,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2637,22 +2782,18 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>CONSUMO DE AGUA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IVA (21%)</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>192298,54</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2668,19 +2809,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J8" s="28">
+      <c r="J8" s="25">
         <f>VALUE(E8)</f>
         <v/>
       </c>
-      <c r="K8" s="28">
+      <c r="K8" s="25">
         <f>IF(D8="IVA (21%)",J8*0.21,0)</f>
         <v/>
       </c>
-      <c r="L8" s="28">
+      <c r="L8" s="25">
         <f>IF(D8="IVA (27%)",J8*0.27,0)</f>
         <v/>
       </c>
-      <c r="M8" s="29">
+      <c r="M8" s="26">
         <f>SUM(J8:L8)</f>
         <v/>
       </c>
@@ -2698,7 +2839,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LA INDIA</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2706,9 +2847,9 @@
           <t>IVA (21%)</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>210533,07</t>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>149955,582505064</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -2729,19 +2870,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J9" s="28">
+      <c r="J9" s="25">
         <f>VALUE(E9)</f>
         <v/>
       </c>
-      <c r="K9" s="28">
+      <c r="K9" s="25">
         <f>IF(D9="IVA (21%)",J9*0.21,0)</f>
         <v/>
       </c>
-      <c r="L9" s="28">
+      <c r="L9" s="25">
         <f>IF(D9="IVA (27%)",J9*0.27,0)</f>
         <v/>
       </c>
-      <c r="M9" s="29">
+      <c r="M9" s="26">
         <f>SUM(J9:L9)</f>
         <v/>
       </c>
@@ -2754,27 +2895,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FOI TERRUÑOS DE LOS ANDES</t>
+          <t>FINCAS Y BODEGAS MONTECHEZ S.A.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AGUA POZO 1</t>
+          <t>LA INDIA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>177077,20</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>543785,298890802</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2790,19 +2931,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J10" s="28">
+      <c r="J10" s="25">
         <f>VALUE(E10)</f>
         <v/>
       </c>
-      <c r="K10" s="28">
+      <c r="K10" s="25">
         <f>IF(D10="IVA (21%)",J10*0.21,0)</f>
         <v/>
       </c>
-      <c r="L10" s="28">
+      <c r="L10" s="25">
         <f>IF(D10="IVA (27%)",J10*0.27,0)</f>
         <v/>
       </c>
-      <c r="M10" s="29">
+      <c r="M10" s="26">
         <f>SUM(J10:L10)</f>
         <v/>
       </c>
@@ -2810,32 +2951,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FOI TERRUÑOS DE LOS ANDES</t>
+          <t>FINCAS Y BODEGAS MONTECHEZ S.A.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AGUA POZO 3</t>
+          <t>POZO 3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="inlineStr">
-        <is>
-          <t>182289,75</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2851,19 +2988,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J11" s="28">
+      <c r="J11" s="25">
         <f>VALUE(E11)</f>
         <v/>
       </c>
-      <c r="K11" s="28">
+      <c r="K11" s="25">
         <f>IF(D11="IVA (21%)",J11*0.21,0)</f>
         <v/>
       </c>
-      <c r="L11" s="28">
+      <c r="L11" s="25">
         <f>IF(D11="IVA (27%)",J11*0.27,0)</f>
         <v/>
       </c>
-      <c r="M11" s="29">
+      <c r="M11" s="26">
         <f>SUM(J11:L11)</f>
         <v/>
       </c>
@@ -2881,7 +3018,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CONSUMO DE AGUA</t>
+          <t>AGUA POZO 1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2889,9 +3026,9 @@
           <t>IVA (27%)</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t>845270,15</t>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>838874,416352994</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2912,19 +3049,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J12" s="28">
+      <c r="J12" s="25">
         <f>VALUE(E12)</f>
         <v/>
       </c>
-      <c r="K12" s="28">
+      <c r="K12" s="25">
         <f>IF(D12="IVA (21%)",J12*0.21,0)</f>
         <v/>
       </c>
-      <c r="L12" s="28">
+      <c r="L12" s="25">
         <f>IF(D12="IVA (27%)",J12*0.27,0)</f>
         <v/>
       </c>
-      <c r="M12" s="29">
+      <c r="M12" s="26">
         <f>SUM(J12:L12)</f>
         <v/>
       </c>
@@ -2942,22 +3079,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>AGUA POZO 3</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IVA (21%)</t>
-        </is>
-      </c>
-      <c r="E13" s="17" t="inlineStr">
-        <is>
-          <t>116029,46</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>1153726,93115259</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2973,19 +3110,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J13" s="28">
+      <c r="J13" s="25">
         <f>VALUE(E13)</f>
         <v/>
       </c>
-      <c r="K13" s="28">
+      <c r="K13" s="25">
         <f>IF(D13="IVA (21%)",J13*0.21,0)</f>
         <v/>
       </c>
-      <c r="L13" s="28">
+      <c r="L13" s="25">
         <f>IF(D13="IVA (27%)",J13*0.27,0)</f>
         <v/>
       </c>
-      <c r="M13" s="29">
+      <c r="M13" s="26">
         <f>SUM(J13:L13)</f>
         <v/>
       </c>
@@ -2993,7 +3130,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3003,22 +3140,18 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LA INDIA</t>
+          <t>CONSUMO DE AGUA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IVA (21%)</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="inlineStr">
-        <is>
-          <t>127031,85</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3034,19 +3167,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J14" s="28">
+      <c r="J14" s="25">
         <f>VALUE(E14)</f>
         <v/>
       </c>
-      <c r="K14" s="28">
+      <c r="K14" s="25">
         <f>IF(D14="IVA (21%)",J14*0.21,0)</f>
         <v/>
       </c>
-      <c r="L14" s="28">
+      <c r="L14" s="25">
         <f>IF(D14="IVA (27%)",J14*0.27,0)</f>
         <v/>
       </c>
-      <c r="M14" s="29">
+      <c r="M14" s="26">
         <f>SUM(J14:L14)</f>
         <v/>
       </c>
@@ -3059,27 +3192,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GRANAR S.A.C y F.</t>
+          <t>FOI TERRUÑOS DE LOS ANDES</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AGUA POZO 1</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>69650,37</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>90480,4909522046</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -3095,19 +3228,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J15" s="28">
+      <c r="J15" s="25">
         <f>VALUE(E15)</f>
         <v/>
       </c>
-      <c r="K15" s="28">
+      <c r="K15" s="25">
         <f>IF(D15="IVA (21%)",J15*0.21,0)</f>
         <v/>
       </c>
-      <c r="L15" s="28">
+      <c r="L15" s="25">
         <f>IF(D15="IVA (27%)",J15*0.27,0)</f>
         <v/>
       </c>
-      <c r="M15" s="29">
+      <c r="M15" s="26">
         <f>SUM(J15:L15)</f>
         <v/>
       </c>
@@ -3120,27 +3253,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GRANAR S.A.C y F.</t>
+          <t>FOI TERRUÑOS DE LOS ANDES</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AGUA POZO 3</t>
+          <t>LA INDIA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E16" s="17" t="inlineStr">
-        <is>
-          <t>71700,63</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>328110,231005036</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3156,19 +3289,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J16" s="28">
+      <c r="J16" s="25">
         <f>VALUE(E16)</f>
         <v/>
       </c>
-      <c r="K16" s="28">
+      <c r="K16" s="25">
         <f>IF(D16="IVA (21%)",J16*0.21,0)</f>
         <v/>
       </c>
-      <c r="L16" s="28">
+      <c r="L16" s="25">
         <f>IF(D16="IVA (27%)",J16*0.27,0)</f>
         <v/>
       </c>
-      <c r="M16" s="29">
+      <c r="M16" s="26">
         <f>SUM(J16:L16)</f>
         <v/>
       </c>
@@ -3176,32 +3309,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GRANAR S.A.C y F.</t>
+          <t>FOI TERRUÑOS DE LOS ANDES</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CONSUMO DE AGUA</t>
+          <t>POZO 1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E17" s="17" t="inlineStr">
-        <is>
-          <t>377594,89</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -3217,19 +3346,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J17" s="28">
+      <c r="J17" s="25">
         <f>VALUE(E17)</f>
         <v/>
       </c>
-      <c r="K17" s="28">
+      <c r="K17" s="25">
         <f>IF(D17="IVA (21%)",J17*0.21,0)</f>
         <v/>
       </c>
-      <c r="L17" s="28">
+      <c r="L17" s="25">
         <f>IF(D17="IVA (27%)",J17*0.27,0)</f>
         <v/>
       </c>
-      <c r="M17" s="29">
+      <c r="M17" s="26">
         <f>SUM(J17:L17)</f>
         <v/>
       </c>
@@ -3247,22 +3376,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>AGUA POZO 1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IVA (21%)</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="inlineStr">
-        <is>
-          <t>56754,78</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>745057,64813477</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3278,19 +3407,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J18" s="28">
+      <c r="J18" s="25">
         <f>VALUE(E18)</f>
         <v/>
       </c>
-      <c r="K18" s="28">
+      <c r="K18" s="25">
         <f>IF(D18="IVA (21%)",J18*0.21,0)</f>
         <v/>
       </c>
-      <c r="L18" s="28">
+      <c r="L18" s="25">
         <f>IF(D18="IVA (27%)",J18*0.27,0)</f>
         <v/>
       </c>
-      <c r="M18" s="29">
+      <c r="M18" s="26">
         <f>SUM(J18:L18)</f>
         <v/>
       </c>
@@ -3308,22 +3437,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LA INDIA</t>
+          <t>AGUA POZO 3</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>IVA (21%)</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="inlineStr">
-        <is>
-          <t>62136,50</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>859343,943989594</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3339,19 +3468,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J19" s="28">
+      <c r="J19" s="25">
         <f>VALUE(E19)</f>
         <v/>
       </c>
-      <c r="K19" s="28">
+      <c r="K19" s="25">
         <f>IF(D19="IVA (21%)",J19*0.21,0)</f>
         <v/>
       </c>
-      <c r="L19" s="28">
+      <c r="L19" s="25">
         <f>IF(D19="IVA (27%)",J19*0.27,0)</f>
         <v/>
       </c>
-      <c r="M19" s="29">
+      <c r="M19" s="26">
         <f>SUM(J19:L19)</f>
         <v/>
       </c>
@@ -3364,12 +3493,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GRANAR S.A.C y F. (AB)</t>
+          <t>GRANAR S.A.C y F.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AGUA POZO 1</t>
+          <t>CONSUMO DE AGUA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3377,10 +3506,10 @@
           <t>IVA (27%)</t>
         </is>
       </c>
-      <c r="E20" s="21" t="n"/>
+      <c r="E20" s="15" t="n"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo: (AB)</t>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3396,19 +3525,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J20" s="28">
+      <c r="J20" s="25">
         <f>VALUE(E20)</f>
         <v/>
       </c>
-      <c r="K20" s="28">
+      <c r="K20" s="25">
         <f>IF(D20="IVA (21%)",J20*0.21,0)</f>
         <v/>
       </c>
-      <c r="L20" s="28">
+      <c r="L20" s="25">
         <f>IF(D20="IVA (27%)",J20*0.27,0)</f>
         <v/>
       </c>
-      <c r="M20" s="29">
+      <c r="M20" s="26">
         <f>SUM(J20:L20)</f>
         <v/>
       </c>
@@ -3416,28 +3545,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GRANAR S.A.C y F. (AB)</t>
+          <t>GRANAR S.A.C y F.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AGUA POZO 3</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E21" s="21" t="n"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo: (AB)</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>44257,7240032306</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3453,19 +3586,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J21" s="28">
+      <c r="J21" s="25">
         <f>VALUE(E21)</f>
         <v/>
       </c>
-      <c r="K21" s="28">
+      <c r="K21" s="25">
         <f>IF(D21="IVA (21%)",J21*0.21,0)</f>
         <v/>
       </c>
-      <c r="L21" s="28">
+      <c r="L21" s="25">
         <f>IF(D21="IVA (27%)",J21*0.27,0)</f>
         <v/>
       </c>
-      <c r="M21" s="29">
+      <c r="M21" s="26">
         <f>SUM(J21:L21)</f>
         <v/>
       </c>
@@ -3478,27 +3611,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GRANAR S.A.C y F. (AB)</t>
+          <t>GRANAR S.A.C y F.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CONSUMO DE AGUA</t>
+          <t>LA INDIA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E22" s="17" t="inlineStr">
-        <is>
-          <t>281861,66</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo: (AB)</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>160492,188908744</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3514,19 +3647,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J22" s="28">
+      <c r="J22" s="25">
         <f>VALUE(E22)</f>
         <v/>
       </c>
-      <c r="K22" s="28">
+      <c r="K22" s="25">
         <f>IF(D22="IVA (21%)",J22*0.21,0)</f>
         <v/>
       </c>
-      <c r="L22" s="28">
+      <c r="L22" s="25">
         <f>IF(D22="IVA (27%)",J22*0.27,0)</f>
         <v/>
       </c>
-      <c r="M22" s="29">
+      <c r="M22" s="26">
         <f>SUM(J22:L22)</f>
         <v/>
       </c>
@@ -3534,17 +3667,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GRANAR S.A.C y F. (AB)</t>
+          <t>GRANAR S.A.C y F.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>POZO 1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3552,14 +3685,10 @@
           <t>IVA (21%)</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
-        <is>
-          <t>69441,14</t>
-        </is>
-      </c>
+      <c r="E23" s="15" t="n"/>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)</t>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3575,19 +3704,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J23" s="28">
+      <c r="J23" s="25">
         <f>VALUE(E23)</f>
         <v/>
       </c>
-      <c r="K23" s="28">
+      <c r="K23" s="25">
         <f>IF(D23="IVA (21%)",J23*0.21,0)</f>
         <v/>
       </c>
-      <c r="L23" s="28">
+      <c r="L23" s="25">
         <f>IF(D23="IVA (27%)",J23*0.27,0)</f>
         <v/>
       </c>
-      <c r="M23" s="29">
+      <c r="M23" s="26">
         <f>SUM(J23:L23)</f>
         <v/>
       </c>
@@ -3605,22 +3734,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LA INDIA</t>
+          <t>AGUA POZO 1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>IVA (21%)</t>
-        </is>
-      </c>
-      <c r="E24" s="17" t="inlineStr">
-        <is>
-          <t>76025,83</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)</t>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>1377109,54533718</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo: (AB)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3636,19 +3765,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J24" s="28">
+      <c r="J24" s="25">
         <f>VALUE(E24)</f>
         <v/>
       </c>
-      <c r="K24" s="28">
+      <c r="K24" s="25">
         <f>IF(D24="IVA (21%)",J24*0.21,0)</f>
         <v/>
       </c>
-      <c r="L24" s="28">
+      <c r="L24" s="25">
         <f>IF(D24="IVA (27%)",J24*0.27,0)</f>
         <v/>
       </c>
-      <c r="M24" s="29">
+      <c r="M24" s="26">
         <f>SUM(J24:L24)</f>
         <v/>
       </c>
@@ -3661,12 +3790,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LLORENTE HNOS SA</t>
+          <t>GRANAR S.A.C y F. (AB)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AGUA POZO 1</t>
+          <t>AGUA POZO 3</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3674,14 +3803,14 @@
           <t>IVA (27%)</t>
         </is>
       </c>
-      <c r="E25" s="17" t="inlineStr">
-        <is>
-          <t>109394,36</t>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>638105,41358851</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo: (AB)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3697,19 +3826,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J25" s="28">
+      <c r="J25" s="25">
         <f>VALUE(E25)</f>
         <v/>
       </c>
-      <c r="K25" s="28">
+      <c r="K25" s="25">
         <f>IF(D25="IVA (21%)",J25*0.21,0)</f>
         <v/>
       </c>
-      <c r="L25" s="28">
+      <c r="L25" s="25">
         <f>IF(D25="IVA (27%)",J25*0.27,0)</f>
         <v/>
       </c>
-      <c r="M25" s="29">
+      <c r="M25" s="26">
         <f>SUM(J25:L25)</f>
         <v/>
       </c>
@@ -3722,12 +3851,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LLORENTE HNOS SA</t>
+          <t>GRANAR S.A.C y F. (AB)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AGUA POZO 3</t>
+          <t>CONSUMO DE AGUA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3735,14 +3864,14 @@
           <t>IVA (27%)</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
-        <is>
-          <t>112614,55</t>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>105002,699462632</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo: (AB)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3758,19 +3887,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J26" s="28">
+      <c r="J26" s="25">
         <f>VALUE(E26)</f>
         <v/>
       </c>
-      <c r="K26" s="28">
+      <c r="K26" s="25">
         <f>IF(D26="IVA (21%)",J26*0.21,0)</f>
         <v/>
       </c>
-      <c r="L26" s="28">
+      <c r="L26" s="25">
         <f>IF(D26="IVA (27%)",J26*0.27,0)</f>
         <v/>
       </c>
-      <c r="M26" s="29">
+      <c r="M26" s="26">
         <f>SUM(J26:L26)</f>
         <v/>
       </c>
@@ -3783,27 +3912,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LLORENTE HNOS SA</t>
+          <t>GRANAR S.A.C y F. (AB)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CONSUMO DE AGUA</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>IVA (27%)</t>
-        </is>
-      </c>
-      <c r="E27" s="17" t="inlineStr">
-        <is>
-          <t>491830,13</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>54150,6270157174</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3819,19 +3948,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J27" s="28">
+      <c r="J27" s="25">
         <f>VALUE(E27)</f>
         <v/>
       </c>
-      <c r="K27" s="28">
+      <c r="K27" s="25">
         <f>IF(D27="IVA (21%)",J27*0.21,0)</f>
         <v/>
       </c>
-      <c r="L27" s="28">
+      <c r="L27" s="25">
         <f>IF(D27="IVA (27%)",J27*0.27,0)</f>
         <v/>
       </c>
-      <c r="M27" s="29">
+      <c r="M27" s="26">
         <f>SUM(J27:L27)</f>
         <v/>
       </c>
@@ -3844,12 +3973,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>LLORENTE HNOS SA</t>
+          <t>GRANAR S.A.C y F. (AB)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>LA INDIA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3857,14 +3986,14 @@
           <t>IVA (21%)</t>
         </is>
       </c>
-      <c r="E28" s="17" t="inlineStr">
-        <is>
-          <t>64201,00</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>196366,913488345</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3880,19 +4009,19 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J28" s="28">
+      <c r="J28" s="25">
         <f>VALUE(E28)</f>
         <v/>
       </c>
-      <c r="K28" s="28">
+      <c r="K28" s="25">
         <f>IF(D28="IVA (21%)",J28*0.21,0)</f>
         <v/>
       </c>
-      <c r="L28" s="28">
+      <c r="L28" s="25">
         <f>IF(D28="IVA (27%)",J28*0.27,0)</f>
         <v/>
       </c>
-      <c r="M28" s="29">
+      <c r="M28" s="26">
         <f>SUM(J28:L28)</f>
         <v/>
       </c>
@@ -3900,17 +4029,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LLORENTE HNOS SA</t>
+          <t>GRANAR S.A.C y F. (AB)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LA INDIA</t>
+          <t>POZO 3</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3918,14 +4047,10 @@
           <t>IVA (21%)</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr">
-        <is>
-          <t>70288,81</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo: (AB)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3941,27 +4066,385 @@
           <t>418001002</t>
         </is>
       </c>
-      <c r="J29" s="28">
+      <c r="J29" s="25">
         <f>VALUE(E29)</f>
         <v/>
       </c>
-      <c r="K29" s="28">
+      <c r="K29" s="25">
         <f>IF(D29="IVA (21%)",J29*0.21,0)</f>
         <v/>
       </c>
-      <c r="L29" s="28">
+      <c r="L29" s="25">
         <f>IF(D29="IVA (27%)",J29*0.27,0)</f>
         <v/>
       </c>
-      <c r="M29" s="29">
+      <c r="M29" s="26">
         <f>SUM(J29:L29)</f>
         <v/>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LLORENTE HNOS SA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>AGUA POZO 1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>652413,021751892</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>418001002</t>
+        </is>
+      </c>
+      <c r="J30" s="25">
+        <f>VALUE(E30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="25">
+        <f>IF(D30="IVA (21%)",J30*0.21,0)</f>
+        <v/>
+      </c>
+      <c r="L30" s="25">
+        <f>IF(D30="IVA (27%)",J30*0.27,0)</f>
+        <v/>
+      </c>
+      <c r="M30" s="26">
+        <f>SUM(J30:L30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>LLORENTE HNOS SA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>AGUA POZO 3</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>768120,023139056</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>418001002</t>
+        </is>
+      </c>
+      <c r="J31" s="25">
+        <f>VALUE(E31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="25">
+        <f>IF(D31="IVA (21%)",J31*0.21,0)</f>
+        <v/>
+      </c>
+      <c r="L31" s="25">
+        <f>IF(D31="IVA (27%)",J31*0.27,0)</f>
+        <v/>
+      </c>
+      <c r="M31" s="26">
+        <f>SUM(J31:L31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>LLORENTE HNOS SA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CONSUMO DE AGUA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>IVA (27%)</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>RECUPERO ENERGIA ELECTRICA Periodo:</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>418001002</t>
+        </is>
+      </c>
+      <c r="J32" s="25">
+        <f>VALUE(E32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="25">
+        <f>IF(D32="IVA (21%)",J32*0.21,0)</f>
+        <v/>
+      </c>
+      <c r="L32" s="25">
+        <f>IF(D32="IVA (27%)",J32*0.27,0)</f>
+        <v/>
+      </c>
+      <c r="M32" s="26">
+        <f>SUM(J32:L32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>LLORENTE HNOS SA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>50064,3373924544</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>418001002</t>
+        </is>
+      </c>
+      <c r="J33" s="25">
+        <f>VALUE(E33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="25">
+        <f>IF(D33="IVA (21%)",J33*0.21,0)</f>
+        <v/>
+      </c>
+      <c r="L33" s="25">
+        <f>IF(D33="IVA (27%)",J33*0.27,0)</f>
+        <v/>
+      </c>
+      <c r="M33" s="26">
+        <f>SUM(J33:L33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>LLORENTE HNOS SA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>LA INDIA</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>181548,764093571</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>418001002</t>
+        </is>
+      </c>
+      <c r="J34" s="25">
+        <f>VALUE(E34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="25">
+        <f>IF(D34="IVA (21%)",J34*0.21,0)</f>
+        <v/>
+      </c>
+      <c r="L34" s="25">
+        <f>IF(D34="IVA (27%)",J34*0.27,0)</f>
+        <v/>
+      </c>
+      <c r="M34" s="26">
+        <f>SUM(J34:L34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>LLORENTE HNOS SA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>POZO 1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>IVA (21%)</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>RENDICIÓN GASTOS FIDEICOMISO Periodo:</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>418001002</t>
+        </is>
+      </c>
+      <c r="J35" s="25">
+        <f>VALUE(E35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="25">
+        <f>IF(D35="IVA (21%)",J35*0.21,0)</f>
+        <v/>
+      </c>
+      <c r="L35" s="25">
+        <f>IF(D35="IVA (27%)",J35*0.27,0)</f>
+        <v/>
+      </c>
+      <c r="M35" s="26">
+        <f>SUM(J35:L35)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M13">
-    <sortState ref="A2:M29">
-      <sortCondition ref="B1:B13"/>
+  <autoFilter ref="A1:M34">
+    <sortState ref="A2:M34">
+      <sortCondition ref="B1:B15"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3974,15 +4457,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B10"/>
+  <dimension ref="A3:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="14.5703125" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15.5703125" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Etiquetas de fila</t>
         </is>
@@ -3994,73 +4477,91 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>CABALGANDO SAFI</t>
         </is>
       </c>
-      <c r="B4" s="30" t="n">
-        <v>2091356.4876</v>
+      <c r="B4" s="27" t="n">
+        <v>25127439.86447715</v>
+      </c>
+      <c r="D4" t="n">
+        <v>25127439</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>FINCAS Y BODEGAS MONTECHEZ S.A.</t>
         </is>
       </c>
-      <c r="B5" s="30" t="n">
-        <v>2027418.1897</v>
+      <c r="B5" s="27" t="n">
+        <v>1764780.15182838</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1764780</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>FOI TERRUÑOS DE LOS ANDES</t>
         </is>
       </c>
-      <c r="B6" s="30" t="n">
-        <v>1823993.3021</v>
+      <c r="B6" s="27" t="n">
+        <v>3037098.484900349</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3037098</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>GRANAR S.A.C y F.</t>
         </is>
       </c>
-      <c r="B7" s="30" t="n">
-        <v>802919.7291</v>
+      <c r="B7" s="27" t="n">
+        <v>2285337.416621432</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2285337</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>GRANAR S.A.C y F. (AB)</t>
         </is>
       </c>
-      <c r="B8" s="30" t="n">
-        <v>533979.3419</v>
+      <c r="B8" s="27" t="n">
+        <v>2995802.650163086</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2995802</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>LLORENTE HNOS SA</t>
         </is>
       </c>
-      <c r="B9" s="30" t="n">
-        <v>1069308.2509</v>
+      <c r="B9" s="27" t="n">
+        <v>2084328.819809595</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2084328</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Total general</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8348975.3013</v>
+        <v>37294787.38779999</v>
       </c>
     </row>
   </sheetData>
@@ -4077,16 +4578,16 @@
   <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
-    <col width="18.7109375" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
-    <col width="9.7109375" bestFit="1" customWidth="1" style="25" min="4" max="4"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
+    <col width="18.7109375" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
+    <col width="9.7109375" bestFit="1" customWidth="1" style="23" min="4" max="4"/>
     <col width="14.5703125" bestFit="1" customWidth="1" style="7" min="5" max="5"/>
-    <col width="16.140625" bestFit="1" customWidth="1" style="25" min="6" max="6"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" style="25" min="7" max="7"/>
-    <col width="10.7109375" bestFit="1" customWidth="1" style="25" min="8" max="8"/>
-    <col width="16.7109375" bestFit="1" customWidth="1" style="25" min="9" max="9"/>
-    <col width="17" bestFit="1" customWidth="1" style="28" min="10" max="10"/>
+    <col width="16.140625" bestFit="1" customWidth="1" style="23" min="6" max="6"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" style="23" min="7" max="7"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="23" min="8" max="8"/>
+    <col width="16.7109375" bestFit="1" customWidth="1" style="23" min="9" max="9"/>
+    <col width="17" bestFit="1" customWidth="1" style="25" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4135,7 +4636,7 @@
           <t>i_cuentaContable</t>
         </is>
       </c>
-      <c r="J1" s="28" t="inlineStr">
+      <c r="J1" s="25" t="inlineStr">
         <is>
           <t>formatoNumero</t>
         </is>
@@ -4229,15 +4730,15 @@
   <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
-    <col width="15.5703125" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
-    <col width="9.7109375" bestFit="1" customWidth="1" style="25" min="4" max="4"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
+    <col width="15.5703125" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
+    <col width="9.7109375" bestFit="1" customWidth="1" style="23" min="4" max="4"/>
     <col width="14" bestFit="1" customWidth="1" style="7" min="5" max="5"/>
-    <col width="14.7109375" bestFit="1" customWidth="1" style="25" min="6" max="6"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" style="25" min="7" max="7"/>
-    <col width="10.7109375" bestFit="1" customWidth="1" style="25" min="8" max="8"/>
-    <col width="16.7109375" bestFit="1" customWidth="1" style="25" min="9" max="9"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" style="23" min="6" max="6"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" style="23" min="7" max="7"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="23" min="8" max="8"/>
+    <col width="16.7109375" bestFit="1" customWidth="1" style="23" min="9" max="9"/>
     <col width="17" bestFit="1" customWidth="1" style="3" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -4287,7 +4788,7 @@
           <t>i_cuentaContable</t>
         </is>
       </c>
-      <c r="J1" s="28" t="inlineStr">
+      <c r="J1" s="25" t="inlineStr">
         <is>
           <t>formatoNumero</t>
         </is>
@@ -4295,49 +4796,49 @@
     </row>
     <row r="2">
       <c r="I2" s="2" t="n"/>
-      <c r="J2" s="28" t="n"/>
+      <c r="J2" s="25" t="n"/>
     </row>
     <row r="3">
       <c r="I3" s="2" t="n"/>
-      <c r="J3" s="28" t="n"/>
+      <c r="J3" s="25" t="n"/>
       <c r="L3" s="11" t="n"/>
     </row>
     <row r="4">
       <c r="I4" s="2" t="n"/>
-      <c r="J4" s="28" t="n"/>
+      <c r="J4" s="25" t="n"/>
       <c r="L4" s="11" t="n"/>
     </row>
     <row r="5">
       <c r="I5" s="2" t="n"/>
-      <c r="J5" s="28" t="n"/>
+      <c r="J5" s="25" t="n"/>
     </row>
     <row r="6">
       <c r="I6" s="2" t="n"/>
-      <c r="J6" s="28" t="n"/>
+      <c r="J6" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="I7" s="2" t="n"/>
-      <c r="J7" s="28" t="n"/>
+      <c r="J7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="I8" s="2" t="n"/>
-      <c r="J8" s="28" t="n"/>
+      <c r="J8" s="25" t="n"/>
     </row>
     <row r="9">
       <c r="I9" s="2" t="n"/>
-      <c r="J9" s="28" t="n"/>
+      <c r="J9" s="25" t="n"/>
     </row>
     <row r="10">
       <c r="I10" s="2" t="n"/>
-      <c r="J10" s="28" t="n"/>
+      <c r="J10" s="25" t="n"/>
     </row>
     <row r="11">
       <c r="I11" s="2" t="n"/>
-      <c r="J11" s="28" t="n"/>
+      <c r="J11" s="25" t="n"/>
     </row>
     <row r="12">
       <c r="I12" s="2" t="n"/>
-      <c r="J12" s="28" t="n"/>
+      <c r="J12" s="25" t="n"/>
     </row>
     <row r="19">
       <c r="C19" s="3" t="n"/>
@@ -4357,15 +4858,15 @@
   <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="22.140625" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
-    <col width="9.7109375" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="22.140625" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
+    <col width="9.7109375" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
     <col width="14" bestFit="1" customWidth="1" style="10" min="4" max="4"/>
-    <col width="20" bestFit="1" customWidth="1" style="25" min="5" max="5"/>
-    <col width="10.28515625" bestFit="1" customWidth="1" style="25" min="6" max="6"/>
-    <col width="10.7109375" bestFit="1" customWidth="1" style="25" min="7" max="7"/>
-    <col width="16.7109375" bestFit="1" customWidth="1" style="25" min="8" max="8"/>
-    <col width="17" bestFit="1" customWidth="1" style="25" min="9" max="9"/>
+    <col width="20" bestFit="1" customWidth="1" style="23" min="5" max="5"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" style="23" min="6" max="6"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="23" min="7" max="7"/>
+    <col width="16.7109375" bestFit="1" customWidth="1" style="23" min="8" max="8"/>
+    <col width="17" bestFit="1" customWidth="1" style="23" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4409,7 +4910,7 @@
           <t>i_cuentaContable</t>
         </is>
       </c>
-      <c r="I1" s="28" t="inlineStr">
+      <c r="I1" s="25" t="inlineStr">
         <is>
           <t>formatoNumero</t>
         </is>
@@ -4418,67 +4919,67 @@
     <row r="2">
       <c r="D2" s="7" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="28" t="n"/>
+      <c r="I2" s="25" t="n"/>
       <c r="K2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="D3" s="7" t="n"/>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" s="28" t="n"/>
+      <c r="I3" s="25" t="n"/>
       <c r="K3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="D4" s="7" t="n"/>
       <c r="H4" s="2" t="n"/>
-      <c r="I4" s="28" t="n"/>
+      <c r="I4" s="25" t="n"/>
       <c r="K4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="D5" s="7" t="n"/>
       <c r="H5" s="2" t="n"/>
-      <c r="I5" s="28" t="n"/>
+      <c r="I5" s="25" t="n"/>
       <c r="K5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="D6" s="7" t="n"/>
       <c r="H6" s="2" t="n"/>
-      <c r="I6" s="28" t="n"/>
+      <c r="I6" s="25" t="n"/>
       <c r="K6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="D7" s="7" t="n"/>
       <c r="H7" s="2" t="n"/>
-      <c r="I7" s="28" t="n"/>
+      <c r="I7" s="25" t="n"/>
       <c r="K7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="D8" s="7" t="n"/>
       <c r="H8" s="2" t="n"/>
-      <c r="I8" s="28" t="n"/>
+      <c r="I8" s="25" t="n"/>
       <c r="K8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="D9" s="7" t="n"/>
       <c r="H9" s="2" t="n"/>
-      <c r="I9" s="28" t="n"/>
+      <c r="I9" s="25" t="n"/>
       <c r="K9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="D10" s="7" t="n"/>
       <c r="H10" s="2" t="n"/>
-      <c r="I10" s="28" t="n"/>
+      <c r="I10" s="25" t="n"/>
       <c r="K10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="D11" s="7" t="n"/>
       <c r="H11" s="2" t="n"/>
-      <c r="I11" s="28" t="n"/>
+      <c r="I11" s="25" t="n"/>
       <c r="K11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="D12" s="7" t="n"/>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="28" t="n"/>
+      <c r="I12" s="25" t="n"/>
       <c r="K12" s="7" t="n"/>
     </row>
   </sheetData>
@@ -4495,13 +4996,13 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col width="33.5703125" bestFit="1" customWidth="1" style="25" min="1" max="1"/>
-    <col width="21.85546875" bestFit="1" customWidth="1" style="25" min="2" max="2"/>
-    <col width="9.7109375" bestFit="1" customWidth="1" style="25" min="3" max="3"/>
+    <col width="33.5703125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
+    <col width="21.85546875" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
+    <col width="9.7109375" bestFit="1" customWidth="1" style="23" min="3" max="3"/>
     <col width="14" bestFit="1" customWidth="1" style="10" min="4" max="4"/>
-    <col width="28.42578125" bestFit="1" customWidth="1" style="25" min="5" max="5"/>
-    <col width="16.7109375" bestFit="1" customWidth="1" style="25" min="8" max="8"/>
-    <col width="17" bestFit="1" customWidth="1" style="25" min="9" max="9"/>
+    <col width="28.42578125" bestFit="1" customWidth="1" style="23" min="5" max="5"/>
+    <col width="16.7109375" bestFit="1" customWidth="1" style="23" min="8" max="8"/>
+    <col width="17" bestFit="1" customWidth="1" style="23" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4545,7 +5046,7 @@
           <t>i_cuentaContable</t>
         </is>
       </c>
-      <c r="I1" s="28" t="inlineStr">
+      <c r="I1" s="25" t="inlineStr">
         <is>
           <t>formatoNumero</t>
         </is>
@@ -4554,42 +5055,42 @@
     <row r="2">
       <c r="E2" s="5" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="28" t="n"/>
+      <c r="I2" s="25" t="n"/>
     </row>
     <row r="3">
       <c r="E3" s="5" t="n"/>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" s="28" t="n"/>
+      <c r="I3" s="25" t="n"/>
     </row>
     <row r="4">
       <c r="E4" s="5" t="n"/>
       <c r="H4" s="2" t="n"/>
-      <c r="I4" s="28" t="n"/>
+      <c r="I4" s="25" t="n"/>
     </row>
     <row r="5">
       <c r="E5" s="5" t="n"/>
       <c r="H5" s="2" t="n"/>
-      <c r="I5" s="28" t="n"/>
+      <c r="I5" s="25" t="n"/>
     </row>
     <row r="6">
       <c r="E6" s="5" t="n"/>
       <c r="H6" s="2" t="n"/>
-      <c r="I6" s="28" t="n"/>
+      <c r="I6" s="25" t="n"/>
     </row>
     <row r="7">
       <c r="E7" s="5" t="n"/>
       <c r="H7" s="2" t="n"/>
-      <c r="I7" s="28" t="n"/>
+      <c r="I7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="E8" s="5" t="n"/>
       <c r="H8" s="2" t="n"/>
-      <c r="I8" s="28" t="n"/>
+      <c r="I8" s="25" t="n"/>
     </row>
     <row r="9">
       <c r="E9" s="5" t="n"/>
       <c r="H9" s="2" t="n"/>
-      <c r="I9" s="28" t="n"/>
+      <c r="I9" s="25" t="n"/>
     </row>
     <row r="21">
       <c r="E21" s="3" t="n"/>

</xml_diff>